<commit_message>
big push on backend cross talk between tabs, new template data and processing of data across all tabs
</commit_message>
<xml_diff>
--- a/www/cost-template.xlsx
+++ b/www/cost-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pathseattle-my.sharepoint.com/personal/hthompson_path_org/Documents/Documents/github/malaria-budgeting-tool/www/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{80C684BE-1432-4728-8906-CC0B9CE4E72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAC33044-4127-4762-9905-AF801A4C0427}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="8_{80C684BE-1432-4728-8906-CC0B9CE4E72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A68DE36-8346-4F92-BBD6-702FF4F5064B}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="7605" yWindow="1215" windowWidth="19860" windowHeight="15420" xr2:uid="{E72D83C0-31FE-469B-BB4E-361133B71EB0}"/>
+    <workbookView xWindow="28845" yWindow="630" windowWidth="21360" windowHeight="16035" activeTab="1" xr2:uid="{E72D83C0-31FE-469B-BB4E-361133B71EB0}"/>
   </bookViews>
   <sheets>
     <sheet name="unit_cost_data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="88">
   <si>
     <t>unit</t>
   </si>
@@ -44,9 +44,6 @@
     <t>cost_class</t>
   </si>
   <si>
-    <t>local_currency_cost</t>
-  </si>
-  <si>
     <t>cm_public</t>
   </si>
   <si>
@@ -207,6 +204,87 @@
   </si>
   <si>
     <t>Standard Pyrethroid</t>
+  </si>
+  <si>
+    <t>per ITN</t>
+  </si>
+  <si>
+    <t>per bale</t>
+  </si>
+  <si>
+    <t>per year</t>
+  </si>
+  <si>
+    <t>per State</t>
+  </si>
+  <si>
+    <t>per LGA</t>
+  </si>
+  <si>
+    <t>per child</t>
+  </si>
+  <si>
+    <t>per dose</t>
+  </si>
+  <si>
+    <t>per facility</t>
+  </si>
+  <si>
+    <t>per SP</t>
+  </si>
+  <si>
+    <t>per AL</t>
+  </si>
+  <si>
+    <t>per RDT kit</t>
+  </si>
+  <si>
+    <t>per RAS</t>
+  </si>
+  <si>
+    <t>per 60mg powder</t>
+  </si>
+  <si>
+    <t>Procurement</t>
+  </si>
+  <si>
+    <t>Distribution</t>
+  </si>
+  <si>
+    <t>Operational</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>Support</t>
+  </si>
+  <si>
+    <t>Net Storage</t>
+  </si>
+  <si>
+    <t>Campaign</t>
+  </si>
+  <si>
+    <t>per SPAQ pack 3-11 month olds</t>
+  </si>
+  <si>
+    <t>per SPAQ pack 12-59 month olds</t>
+  </si>
+  <si>
+    <t>ngn_cost</t>
+  </si>
+  <si>
+    <t>AL</t>
+  </si>
+  <si>
+    <t>Artesunate injections</t>
+  </si>
+  <si>
+    <t>RAS</t>
+  </si>
+  <si>
+    <t>RDT kits</t>
   </si>
 </sst>
 </file>
@@ -690,8 +768,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1067,40 +1146,422 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6649CC70-95E1-4A45-9BAC-E2E83642FF0B}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="21.42578125" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="8" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>7</v>
       </c>
-      <c r="F1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
+      <c r="B21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C21" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>86</v>
+      </c>
+      <c r="C26" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1112,7 +1573,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2B23E79F-74DE-47A3-AA72-02125CE1366C}">
           <x14:formula1>
             <xm:f>'list-items-ignore'!$B$1:$B$10</xm:f>
@@ -1121,9 +1582,15 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5E138DD-4BA1-445F-A665-4841EF8F02BE}">
           <x14:formula1>
-            <xm:f>'list-items-ignore'!$D$1:$D$44</xm:f>
+            <xm:f>'list-items-ignore'!$D:$D</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{613C0C3E-E487-435C-8D59-412773A42907}">
+          <x14:formula1>
+            <xm:f>'list-items-ignore'!$G:$G</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1133,257 +1600,332 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{329D48F2-0C03-4D47-B72E-EFAD5BE6EF6C}">
-  <dimension ref="B1:D44"/>
+  <dimension ref="B1:G50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+      <c r="G2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="G3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+      <c r="G4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="G5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
+      <c r="G6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
+      <c r="G7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+      <c r="G8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
         <v>15</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
+      <c r="G9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D10" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="G10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D11" t="s">
+      <c r="G11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D12" t="s">
+      <c r="G12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D13" t="s">
+      <c r="G13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D14" t="s">
+      <c r="G14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D15" t="s">
+      <c r="G15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D16" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="17" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="39" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="40" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="41" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="42" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D42" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="43" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D44" t="s">
-        <v>61</v>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D45" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D46" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="48" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D48" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D49" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="50" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D50" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FR version of DRC specific demo instance
</commit_message>
<xml_diff>
--- a/www/cost-template.xlsx
+++ b/www/cost-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pathseattle-my.sharepoint.com/personal/hthompson_path_org/Documents/Documents/github/malaria-budgeting-tool/www/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="8_{80C684BE-1432-4728-8906-CC0B9CE4E72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A68DE36-8346-4F92-BBD6-702FF4F5064B}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="8_{80C684BE-1432-4728-8906-CC0B9CE4E72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B8C6A23-0949-41A1-A135-866A801AC0F1}"/>
   <bookViews>
-    <workbookView xWindow="28845" yWindow="630" windowWidth="21360" windowHeight="16035" activeTab="1" xr2:uid="{E72D83C0-31FE-469B-BB4E-361133B71EB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E72D83C0-31FE-469B-BB4E-361133B71EB0}"/>
   </bookViews>
   <sheets>
     <sheet name="unit_cost_data" sheetId="1" r:id="rId1"/>
@@ -272,9 +272,6 @@
     <t>per SPAQ pack 12-59 month olds</t>
   </si>
   <si>
-    <t>ngn_cost</t>
-  </si>
-  <si>
     <t>AL</t>
   </si>
   <si>
@@ -285,6 +282,9 @@
   </si>
   <si>
     <t>RDT kits</t>
+  </si>
+  <si>
+    <t>local_currency</t>
   </si>
 </sst>
 </file>
@@ -1172,7 +1172,7 @@
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -1449,7 +1449,7 @@
         <v>7</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C21" t="s">
         <v>74</v>
@@ -1463,7 +1463,7 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C22" t="s">
         <v>75</v>
@@ -1477,7 +1477,7 @@
         <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C23" t="s">
         <v>74</v>
@@ -1491,7 +1491,7 @@
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C24" t="s">
         <v>75</v>
@@ -1505,7 +1505,7 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C25" t="s">
         <v>74</v>
@@ -1519,7 +1519,7 @@
         <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C26" t="s">
         <v>75</v>
@@ -1533,7 +1533,7 @@
         <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
         <v>74</v>
@@ -1547,7 +1547,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C28" t="s">
         <v>75</v>
@@ -1910,22 +1910,22 @@
     </row>
     <row r="47" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D47" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D48" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="49" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D49" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="50" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D50" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>